<commit_message>
Product Book: planta estrutural, fachada traseira, renders web, exportação PDF e versão autônoma
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MXgeeezmv3d1TAAP83TAQH
</commit_message>
<xml_diff>
--- a/projects/zion-glamping-line/ZION_ORCAMENTO_SC_Cocoon_Zenith.xlsx
+++ b/projects/zion-glamping-line/ZION_ORCAMENTO_SC_Cocoon_Zenith.xlsx
@@ -4350,13 +4350,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>389685.716</v>
+        <v>389685.72</v>
       </c>
       <c r="C2" t="n">
         <v>563565</v>
       </c>
       <c r="D2" t="n">
-        <v>775639.4440000001</v>
+        <v>775639.4399999999</v>
       </c>
     </row>
     <row r="3">
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>61261.19999999999</v>
+        <v>61261.2</v>
       </c>
       <c r="C4" t="n">
         <v>68068</v>
@@ -4462,13 +4462,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>254818.996</v>
+        <v>254819</v>
       </c>
       <c r="C9" t="n">
         <v>327744</v>
       </c>
       <c r="D9" t="n">
-        <v>435556.3540000002</v>
+        <v>435556.35</v>
       </c>
     </row>
     <row r="10">
@@ -4478,13 +4478,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>59941.95791999999</v>
+        <v>59941.96</v>
       </c>
       <c r="C10" t="n">
         <v>81874.56</v>
       </c>
       <c r="D10" t="n">
-        <v>108568.56528</v>
+        <v>108568.57</v>
       </c>
     </row>
     <row r="11">
@@ -4494,13 +4494,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>49951.63159999999</v>
+        <v>49951.63</v>
       </c>
       <c r="C11" t="n">
         <v>54583.04</v>
       </c>
       <c r="D11" t="n">
-        <v>72379.04352000002</v>
+        <v>72379.03999999999</v>
       </c>
     </row>
     <row r="12">
@@ -4526,13 +4526,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>849409.9055199999</v>
+        <v>849409.91</v>
       </c>
       <c r="C13" t="n">
         <v>1058745.6</v>
       </c>
       <c r="D13" t="n">
-        <v>1325685.6528</v>
+        <v>1325685.65</v>
       </c>
     </row>
     <row r="14">
@@ -4542,13 +4542,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>609409.9055199999</v>
+        <v>609409.91</v>
       </c>
       <c r="C14" t="n">
-        <v>818745.6000000001</v>
+        <v>818745.6</v>
       </c>
       <c r="D14" t="n">
-        <v>1085685.6528</v>
+        <v>1085685.65</v>
       </c>
     </row>
     <row r="15">
@@ -4558,13 +4558,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10711.34811500631</v>
+        <v>10711.35</v>
       </c>
       <c r="C15" t="n">
-        <v>13351.14249684742</v>
+        <v>13351.14</v>
       </c>
       <c r="D15" t="n">
-        <v>16717.34745018916</v>
+        <v>16717.35</v>
       </c>
     </row>
     <row r="16">
@@ -4574,13 +4574,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>17549.79143636363</v>
+        <v>17549.79</v>
       </c>
       <c r="C16" t="n">
-        <v>21874.90909090909</v>
+        <v>21874.91</v>
       </c>
       <c r="D16" t="n">
-        <v>27390.19943801653</v>
+        <v>27390.2</v>
       </c>
     </row>
   </sheetData>
@@ -4672,7 +4672,7 @@
         <v>1058745.6</v>
       </c>
       <c r="H2" t="n">
-        <v>13351.14249684742</v>
+        <v>13351.14</v>
       </c>
     </row>
     <row r="3">
@@ -4689,16 +4689,16 @@
         <v>29151</v>
       </c>
       <c r="E3" t="n">
-        <v>108823.9632</v>
+        <v>108823.96</v>
       </c>
       <c r="F3" t="n">
         <v>48000</v>
       </c>
       <c r="G3" t="n">
-        <v>796964.9232</v>
+        <v>796964.92</v>
       </c>
       <c r="H3" t="n">
-        <v>10049.99903152585</v>
+        <v>10050</v>
       </c>
     </row>
     <row r="4">
@@ -4715,16 +4715,16 @@
         <v>27165.25</v>
       </c>
       <c r="E4" t="n">
-        <v>92082.3645</v>
+        <v>92082.36</v>
       </c>
       <c r="F4" t="n">
         <v>24000</v>
       </c>
       <c r="G4" t="n">
-        <v>729964.7945</v>
+        <v>729964.79</v>
       </c>
       <c r="H4" t="n">
-        <v>9205.104596469104</v>
+        <v>9205.1</v>
       </c>
     </row>
     <row r="5">
@@ -4735,22 +4735,22 @@
         <v>480957.01</v>
       </c>
       <c r="C5" t="n">
-        <v>65925.20000000001</v>
+        <v>65925.2</v>
       </c>
       <c r="D5" t="n">
         <v>24256</v>
       </c>
       <c r="E5" t="n">
-        <v>74247.96729999999</v>
+        <v>74247.97</v>
       </c>
       <c r="F5" t="n">
         <v>4800</v>
       </c>
       <c r="G5" t="n">
-        <v>650186.1773</v>
+        <v>650186.1800000001</v>
       </c>
       <c r="H5" t="n">
-        <v>8199.069070617907</v>
+        <v>8199.07</v>
       </c>
     </row>
   </sheetData>
@@ -9718,13 +9718,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>354374.478</v>
+        <v>354374.48</v>
       </c>
       <c r="C2" t="n">
         <v>500452.4</v>
       </c>
       <c r="D2" t="n">
-        <v>676363.782</v>
+        <v>676363.78</v>
       </c>
     </row>
     <row r="3">
@@ -9830,13 +9830,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>217208.718</v>
+        <v>217208.72</v>
       </c>
       <c r="C9" t="n">
         <v>276713.8</v>
       </c>
       <c r="D9" t="n">
-        <v>359977.832</v>
+        <v>359977.83</v>
       </c>
     </row>
     <row r="10">
@@ -9846,13 +9846,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>53609.08775999999</v>
+        <v>53609.09</v>
       </c>
       <c r="C10" t="n">
-        <v>72080.54399999999</v>
+        <v>72080.53999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>94274.50343999999</v>
+        <v>94274.5</v>
       </c>
     </row>
     <row r="11">
@@ -9862,13 +9862,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>44674.2398</v>
+        <v>44674.24</v>
       </c>
       <c r="C11" t="n">
-        <v>48053.696</v>
+        <v>48053.7</v>
       </c>
       <c r="D11" t="n">
-        <v>62849.66896</v>
+        <v>62849.67</v>
       </c>
     </row>
     <row r="12">
@@ -9894,13 +9894,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>785025.7255599999</v>
+        <v>785025.73</v>
       </c>
       <c r="C13" t="n">
         <v>960805.4399999999</v>
       </c>
       <c r="D13" t="n">
-        <v>1182745.0344</v>
+        <v>1182745.03</v>
       </c>
     </row>
     <row r="14">
@@ -9910,13 +9910,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>545025.7255599999</v>
+        <v>545025.73</v>
       </c>
       <c r="C14" t="n">
         <v>720805.4399999999</v>
       </c>
       <c r="D14" t="n">
-        <v>942745.0344</v>
+        <v>942745.03</v>
       </c>
     </row>
     <row r="15">
@@ -9926,13 +9926,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10064.43237897436</v>
+        <v>10064.43</v>
       </c>
       <c r="C15" t="n">
-        <v>12318.01846153846</v>
+        <v>12318.02</v>
       </c>
       <c r="D15" t="n">
-        <v>15163.39787692308</v>
+        <v>15163.4</v>
       </c>
     </row>
     <row r="16">
@@ -9942,13 +9942,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>16354.70261583333</v>
+        <v>16354.7</v>
       </c>
       <c r="C16" t="n">
         <v>20016.78</v>
       </c>
       <c r="D16" t="n">
-        <v>24640.52155</v>
+        <v>24640.52</v>
       </c>
     </row>
   </sheetData>
@@ -10040,7 +10040,7 @@
         <v>960805.4399999999</v>
       </c>
       <c r="H2" t="n">
-        <v>12318.01846153846</v>
+        <v>12318.02</v>
       </c>
     </row>
     <row r="3">
@@ -10051,22 +10051,22 @@
         <v>474062.96</v>
       </c>
       <c r="C3" t="n">
-        <v>67482.296</v>
+        <v>67482.3</v>
       </c>
       <c r="D3" t="n">
         <v>22668</v>
       </c>
       <c r="E3" t="n">
-        <v>95916.25352000003</v>
+        <v>95916.25</v>
       </c>
       <c r="F3" t="n">
         <v>48000</v>
       </c>
       <c r="G3" t="n">
-        <v>708129.5095200001</v>
+        <v>708129.51</v>
       </c>
       <c r="H3" t="n">
-        <v>9078.583455384616</v>
+        <v>9078.58</v>
       </c>
     </row>
     <row r="4">
@@ -10074,25 +10074,25 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>457113.568</v>
+        <v>457113.57</v>
       </c>
       <c r="C4" t="n">
-        <v>63167.85599999999</v>
+        <v>63167.86</v>
       </c>
       <c r="D4" t="n">
         <v>21221</v>
       </c>
       <c r="E4" t="n">
-        <v>81225.3636</v>
+        <v>81225.36</v>
       </c>
       <c r="F4" t="n">
         <v>24000</v>
       </c>
       <c r="G4" t="n">
-        <v>646727.7876</v>
+        <v>646727.79</v>
       </c>
       <c r="H4" t="n">
-        <v>8291.381892307692</v>
+        <v>8291.379999999999</v>
       </c>
     </row>
     <row r="5">
@@ -10100,25 +10100,25 @@
         <v>50</v>
       </c>
       <c r="B5" t="n">
-        <v>428284.388</v>
+        <v>428284.39</v>
       </c>
       <c r="C5" t="n">
-        <v>56972.04000000001</v>
+        <v>56972.04</v>
       </c>
       <c r="D5" t="n">
         <v>19106</v>
       </c>
       <c r="E5" t="n">
-        <v>65567.11564</v>
+        <v>65567.12</v>
       </c>
       <c r="F5" t="n">
         <v>4800</v>
       </c>
       <c r="G5" t="n">
-        <v>574729.5436399999</v>
+        <v>574729.54</v>
       </c>
       <c r="H5" t="n">
-        <v>7368.327482564102</v>
+        <v>7368.33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Product Book final: modelos explodidos, camadas construtivas, PDFs e versão autônoma regenerados; contagem de estacas alinhada (44)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MXgeeezmv3d1TAAP83TAQH
</commit_message>
<xml_diff>
--- a/projects/zion-glamping-line/ZION_ORCAMENTO_SC_Cocoon_Zenith.xlsx
+++ b/projects/zion-glamping-line/ZION_ORCAMENTO_SC_Cocoon_Zenith.xlsx
@@ -2991,7 +2991,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D42" t="n">
         <v>0.15</v>
@@ -3019,7 +3019,7 @@
         <v>1.4</v>
       </c>
       <c r="K42" t="n">
-        <v>64.40000000000001</v>
+        <v>61.6</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D54" t="n">
         <v>2</v>
@@ -3751,7 +3751,7 @@
         <v>18.4</v>
       </c>
       <c r="K54" t="n">
-        <v>845.5</v>
+        <v>808.7</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
@@ -3784,7 +3784,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D55" t="n">
         <v>0.25</v>
@@ -3812,7 +3812,7 @@
         <v>2.2</v>
       </c>
       <c r="K55" t="n">
-        <v>101.2</v>
+        <v>96.8</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
@@ -6654,7 +6654,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G2" t="n">
         <v>2</v>
@@ -6687,7 +6687,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="G3" t="n">
         <v>3</v>
@@ -7524,25 +7524,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E4" t="n">
         <v>9.119999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>1960.8</v>
+        <v>1933.44</v>
       </c>
       <c r="G4" t="n">
         <v>9.6</v>
       </c>
       <c r="H4" t="n">
-        <v>2064</v>
+        <v>2035.2</v>
       </c>
       <c r="I4" t="n">
         <v>10.08</v>
       </c>
       <c r="J4" t="n">
-        <v>2167.2</v>
+        <v>2136.96</v>
       </c>
     </row>
     <row r="5">
@@ -7562,25 +7562,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1343</v>
+        <v>1340</v>
       </c>
       <c r="E5" t="n">
         <v>5.6</v>
       </c>
       <c r="F5" t="n">
-        <v>7520.8</v>
+        <v>7504</v>
       </c>
       <c r="G5" t="n">
         <v>7.4</v>
       </c>
       <c r="H5" t="n">
-        <v>9938.200000000001</v>
+        <v>9916</v>
       </c>
       <c r="I5" t="n">
         <v>7.4</v>
       </c>
       <c r="J5" t="n">
-        <v>9938.200000000001</v>
+        <v>9916</v>
       </c>
     </row>
     <row r="6">
@@ -7600,7 +7600,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -7612,13 +7612,13 @@
         <v>4.9</v>
       </c>
       <c r="H6" t="n">
-        <v>4606</v>
+        <v>4596.2</v>
       </c>
       <c r="I6" t="n">
         <v>5.63</v>
       </c>
       <c r="J6" t="n">
-        <v>5296.9</v>
+        <v>5285.63</v>
       </c>
     </row>
     <row r="7">
@@ -8550,25 +8550,25 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E31" t="n">
         <v>576</v>
       </c>
       <c r="F31" t="n">
-        <v>26496</v>
+        <v>25344</v>
       </c>
       <c r="G31" t="n">
         <v>640</v>
       </c>
       <c r="H31" t="n">
-        <v>29440</v>
+        <v>28160</v>
       </c>
       <c r="I31" t="n">
         <v>672</v>
       </c>
       <c r="J31" t="n">
-        <v>30912</v>
+        <v>29568</v>
       </c>
     </row>
     <row r="32">
@@ -8588,25 +8588,25 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E32" t="n">
         <v>256.5</v>
       </c>
       <c r="F32" t="n">
-        <v>11799</v>
+        <v>11286</v>
       </c>
       <c r="G32" t="n">
         <v>270</v>
       </c>
       <c r="H32" t="n">
-        <v>12420</v>
+        <v>11880</v>
       </c>
       <c r="I32" t="n">
         <v>270</v>
       </c>
       <c r="J32" t="n">
-        <v>12420</v>
+        <v>11880</v>
       </c>
     </row>
     <row r="33">
@@ -9190,15 +9190,15 @@
       <c r="D48" s="2" t="inlineStr"/>
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="n">
-        <v>354374.478</v>
+        <v>352665.318</v>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="n">
-        <v>500452.4</v>
+        <v>498571.6</v>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="n">
-        <v>676363.782</v>
+        <v>674416.072</v>
       </c>
     </row>
   </sheetData>
@@ -9718,13 +9718,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>354374.48</v>
+        <v>352665.32</v>
       </c>
       <c r="C2" t="n">
-        <v>500452.4</v>
+        <v>498571.6</v>
       </c>
       <c r="D2" t="n">
-        <v>676363.78</v>
+        <v>674416.0699999999</v>
       </c>
     </row>
     <row r="3">
@@ -9814,13 +9814,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>229533.68</v>
+        <v>229489.52</v>
       </c>
       <c r="C8" t="n">
-        <v>323957.4</v>
+        <v>323896.6</v>
       </c>
       <c r="D8" t="n">
-        <v>425643.03</v>
+        <v>425579.32</v>
       </c>
     </row>
     <row r="9">
@@ -9830,13 +9830,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>217208.72</v>
+        <v>215543.72</v>
       </c>
       <c r="C9" t="n">
-        <v>276713.8</v>
+        <v>274893.8</v>
       </c>
       <c r="D9" t="n">
-        <v>359977.83</v>
+        <v>358093.83</v>
       </c>
     </row>
     <row r="10">
@@ -9846,13 +9846,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>53609.09</v>
+        <v>53403.99</v>
       </c>
       <c r="C10" t="n">
-        <v>72080.53999999999</v>
+        <v>71854.85000000001</v>
       </c>
       <c r="D10" t="n">
-        <v>94274.5</v>
+        <v>94040.78</v>
       </c>
     </row>
     <row r="11">
@@ -9862,13 +9862,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>44674.24</v>
+        <v>44503.32</v>
       </c>
       <c r="C11" t="n">
-        <v>48053.7</v>
+        <v>47903.23</v>
       </c>
       <c r="D11" t="n">
-        <v>62849.67</v>
+        <v>62693.85</v>
       </c>
     </row>
     <row r="12">
@@ -9894,13 +9894,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>785025.73</v>
+        <v>782940.55</v>
       </c>
       <c r="C13" t="n">
-        <v>960805.4399999999</v>
+        <v>958548.48</v>
       </c>
       <c r="D13" t="n">
-        <v>1182745.03</v>
+        <v>1180407.78</v>
       </c>
     </row>
     <row r="14">
@@ -9910,13 +9910,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>545025.73</v>
+        <v>542940.55</v>
       </c>
       <c r="C14" t="n">
-        <v>720805.4399999999</v>
+        <v>718548.48</v>
       </c>
       <c r="D14" t="n">
-        <v>942745.03</v>
+        <v>940407.78</v>
       </c>
     </row>
     <row r="15">
@@ -9926,13 +9926,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10064.43</v>
+        <v>10037.7</v>
       </c>
       <c r="C15" t="n">
-        <v>12318.02</v>
+        <v>12289.08</v>
       </c>
       <c r="D15" t="n">
-        <v>15163.4</v>
+        <v>15133.43</v>
       </c>
     </row>
     <row r="16">
@@ -9942,13 +9942,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>16354.7</v>
+        <v>16311.26</v>
       </c>
       <c r="C16" t="n">
-        <v>20016.78</v>
+        <v>19969.76</v>
       </c>
       <c r="D16" t="n">
-        <v>24640.52</v>
+        <v>24591.83</v>
       </c>
     </row>
   </sheetData>
@@ -10022,7 +10022,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>500452.4</v>
+        <v>498571.6</v>
       </c>
       <c r="C2" t="n">
         <v>74618.8</v>
@@ -10031,16 +10031,16 @@
         <v>25600</v>
       </c>
       <c r="E2" t="n">
-        <v>120134.24</v>
+        <v>119758.08</v>
       </c>
       <c r="F2" t="n">
         <v>240000</v>
       </c>
       <c r="G2" t="n">
-        <v>960805.4399999999</v>
+        <v>958548.48</v>
       </c>
       <c r="H2" t="n">
-        <v>12318.02</v>
+        <v>12289.08</v>
       </c>
     </row>
     <row r="3">
@@ -10048,7 +10048,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>474062.96</v>
+        <v>472276.2</v>
       </c>
       <c r="C3" t="n">
         <v>67482.3</v>
@@ -10057,16 +10057,16 @@
         <v>22668</v>
       </c>
       <c r="E3" t="n">
-        <v>95916.25</v>
+        <v>95612.5</v>
       </c>
       <c r="F3" t="n">
         <v>48000</v>
       </c>
       <c r="G3" t="n">
-        <v>708129.51</v>
+        <v>706039</v>
       </c>
       <c r="H3" t="n">
-        <v>9078.58</v>
+        <v>9051.780000000001</v>
       </c>
     </row>
     <row r="4">
@@ -10074,7 +10074,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>457113.57</v>
+        <v>455383.23</v>
       </c>
       <c r="C4" t="n">
         <v>63167.86</v>
@@ -10083,16 +10083,16 @@
         <v>21221</v>
       </c>
       <c r="E4" t="n">
-        <v>81225.36</v>
+        <v>80965.81</v>
       </c>
       <c r="F4" t="n">
         <v>24000</v>
       </c>
       <c r="G4" t="n">
-        <v>646727.79</v>
+        <v>644737.9</v>
       </c>
       <c r="H4" t="n">
-        <v>8291.379999999999</v>
+        <v>8265.870000000001</v>
       </c>
     </row>
     <row r="5">
@@ -10100,7 +10100,7 @@
         <v>50</v>
       </c>
       <c r="B5" t="n">
-        <v>428284.39</v>
+        <v>426629.89</v>
       </c>
       <c r="C5" t="n">
         <v>56972.04</v>
@@ -10109,16 +10109,16 @@
         <v>19106</v>
       </c>
       <c r="E5" t="n">
-        <v>65567.12</v>
+        <v>65352.03</v>
       </c>
       <c r="F5" t="n">
         <v>4800</v>
       </c>
       <c r="G5" t="n">
-        <v>574729.54</v>
+        <v>572859.96</v>
       </c>
       <c r="H5" t="n">
-        <v>7368.33</v>
+        <v>7344.36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>